<commit_message>
Protection anti-coupure de courant, pause/reprise auto Internet, sauvegarde Excel au fil de l'eau et AutoUpdater GitHub
</commit_message>
<xml_diff>
--- a/dossiers.xlsx
+++ b/dossiers.xlsx
@@ -601,6 +601,11 @@
           <t>VV1819</t>
         </is>
       </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -608,6 +613,11 @@
           <t>VV1820</t>
         </is>
       </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -615,6 +625,11 @@
           <t>VV1822</t>
         </is>
       </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -622,6 +637,11 @@
           <t>VV1824</t>
         </is>
       </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -629,6 +649,11 @@
           <t>VV1828</t>
         </is>
       </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -636,6 +661,11 @@
           <t>VV1830</t>
         </is>
       </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -643,6 +673,11 @@
           <t>VV1831</t>
         </is>
       </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -650,6 +685,11 @@
           <t>VV1832</t>
         </is>
       </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -657,11 +697,21 @@
           <t>VV1844</t>
         </is>
       </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
           <t>VV1846</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Intégration complète du pack d'identité visuelle et de la charte graphique v1.0 (v1.3.0)
</commit_message>
<xml_diff>
--- a/dossiers.xlsx
+++ b/dossiers.xlsx
@@ -721,6 +721,11 @@
           <t>VV1848</t>
         </is>
       </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -728,6 +733,11 @@
           <t>VV1849</t>
         </is>
       </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -735,6 +745,11 @@
           <t>VV1850</t>
         </is>
       </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -742,6 +757,11 @@
           <t>VV1851</t>
         </is>
       </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -749,6 +769,11 @@
           <t>VV1852</t>
         </is>
       </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -756,6 +781,11 @@
           <t>VV1853</t>
         </is>
       </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -770,6 +800,11 @@
           <t>VV1855</t>
         </is>
       </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -777,6 +812,11 @@
           <t>VV1858</t>
         </is>
       </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -784,6 +824,11 @@
           <t>VV1859</t>
         </is>
       </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -791,6 +836,11 @@
           <t>VV1860</t>
         </is>
       </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -798,6 +848,11 @@
           <t>VV1861</t>
         </is>
       </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -805,6 +860,11 @@
           <t>VV1862</t>
         </is>
       </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -812,6 +872,11 @@
           <t>VV1864</t>
         </is>
       </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -819,6 +884,11 @@
           <t>VV1865</t>
         </is>
       </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -826,6 +896,11 @@
           <t>VV1867</t>
         </is>
       </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -833,6 +908,11 @@
           <t>VV1870</t>
         </is>
       </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -840,6 +920,11 @@
           <t>VV1874</t>
         </is>
       </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -847,6 +932,11 @@
           <t>VV1875</t>
         </is>
       </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -854,11 +944,21 @@
           <t>VV1876</t>
         </is>
       </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
           <t>VV1877</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correction de l'icône officielle dans la barre des tâches Windows, la barre de titre, le .exe et le Bureau (v1.3.1)
</commit_message>
<xml_diff>
--- a/dossiers.xlsx
+++ b/dossiers.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +33,14 @@
     <font>
       <b val="1"/>
       <color rgb="00107C41"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000878F9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0016A34A"/>
     </font>
   </fonts>
   <fills count="3">
@@ -61,12 +69,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -968,6 +978,11 @@
           <t>VV1878</t>
         </is>
       </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -975,6 +990,11 @@
           <t>VV1883</t>
         </is>
       </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -982,6 +1002,11 @@
           <t>VV1884</t>
         </is>
       </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -989,6 +1014,11 @@
           <t>VV1885</t>
         </is>
       </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -996,6 +1026,11 @@
           <t>VV1886</t>
         </is>
       </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1003,6 +1038,11 @@
           <t>VV1887</t>
         </is>
       </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1010,6 +1050,11 @@
           <t>VV1889</t>
         </is>
       </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1017,6 +1062,11 @@
           <t>VV1890</t>
         </is>
       </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1024,6 +1074,11 @@
           <t>VV1891</t>
         </is>
       </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1031,6 +1086,11 @@
           <t>VV1892</t>
         </is>
       </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1038,6 +1098,11 @@
           <t>VV1893</t>
         </is>
       </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1045,6 +1110,11 @@
           <t>VV1894</t>
         </is>
       </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1052,6 +1122,11 @@
           <t>VV1895</t>
         </is>
       </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1059,11 +1134,21 @@
           <t>VV1896</t>
         </is>
       </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
           <t>VV1902</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>En cours</t>
         </is>
       </c>
     </row>

</xml_diff>